<commit_message>
docs(training-trend-analyzer): localize publication dashboard view
</commit_message>
<xml_diff>
--- a/training-trend-analyzer/ops/publication_dashboard/publication_weekly_view.xlsx
+++ b/training-trend-analyzer/ops/publication_dashboard/publication_weekly_view.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Weekly_Overview" sheetId="1" r:id="rId1"/>
-    <sheet name="Coverage_Check" sheetId="2" r:id="rId2"/>
-    <sheet name="Release_Log" sheetId="3" r:id="rId3"/>
+    <sheet name="週次概要" sheetId="1" r:id="rId1"/>
+    <sheet name="充足確認" sheetId="2" r:id="rId2"/>
+    <sheet name="公開履歴" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -64,57 +64,57 @@
       </c>
       <c r="C1" t="inlineStr" s="1">
         <is>
-          <t>publish_ready</t>
+          <t>公開準備OK</t>
         </is>
       </c>
       <c r="D1" t="inlineStr" s="1">
         <is>
-          <t>content_kind</t>
+          <t>公開種別</t>
         </is>
       </c>
       <c r="E1" t="inlineStr" s="1">
         <is>
-          <t>GT coverage</t>
+          <t>GT充足</t>
         </is>
       </c>
       <c r="F1" t="inlineStr" s="1">
         <is>
-          <t>GS coverage</t>
+          <t>GS充足</t>
         </is>
       </c>
       <c r="G1" t="inlineStr" s="1">
         <is>
-          <t>YT coverage</t>
+          <t>YT充足</t>
         </is>
       </c>
       <c r="H1" t="inlineStr" s="1">
         <is>
-          <t>ranking review</t>
+          <t>ランキング確認</t>
         </is>
       </c>
       <c r="I1" t="inlineStr" s="1">
         <is>
-          <t>ranking release</t>
+          <t>ランキング公開</t>
         </is>
       </c>
       <c r="J1" t="inlineStr" s="1">
         <is>
-          <t>compare review</t>
+          <t>比較確認</t>
         </is>
       </c>
       <c r="K1" t="inlineStr" s="1">
         <is>
-          <t>compare release</t>
+          <t>比較公開</t>
         </is>
       </c>
       <c r="L1" t="inlineStr" s="1">
         <is>
-          <t>verify all</t>
+          <t>全体検証</t>
         </is>
       </c>
       <c r="M1" t="inlineStr" s="1">
         <is>
-          <t>handoff</t>
+          <t>引継ぎファイル</t>
         </is>
       </c>
       <c r="N1" t="inlineStr" s="1">
@@ -141,17 +141,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>完了</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>はい</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ranking / compare closed</t>
+          <t>ランキング・比較とも完了</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -171,27 +171,27 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>完了</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>完了</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>完了</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>完了</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -238,47 +238,47 @@
       </c>
       <c r="C1" t="inlineStr" s="1">
         <is>
-          <t>GT present</t>
+          <t>GT取得済み</t>
         </is>
       </c>
       <c r="D1" t="inlineStr" s="1">
         <is>
-          <t>GT missing</t>
+          <t>GT不足</t>
         </is>
       </c>
       <c r="E1" t="inlineStr" s="1">
         <is>
-          <t>GT coverage率</t>
+          <t>GT充足率</t>
         </is>
       </c>
       <c r="F1" t="inlineStr" s="1">
         <is>
-          <t>GS present</t>
+          <t>GS取得済み</t>
         </is>
       </c>
       <c r="G1" t="inlineStr" s="1">
         <is>
-          <t>GS missing</t>
+          <t>GS不足</t>
         </is>
       </c>
       <c r="H1" t="inlineStr" s="1">
         <is>
-          <t>GS coverage率</t>
+          <t>GS充足率</t>
         </is>
       </c>
       <c r="I1" t="inlineStr" s="1">
         <is>
-          <t>YT present</t>
+          <t>YT取得済み</t>
         </is>
       </c>
       <c r="J1" t="inlineStr" s="1">
         <is>
-          <t>YT missing</t>
+          <t>YT不足</t>
         </is>
       </c>
       <c r="K1" t="inlineStr" s="1">
         <is>
-          <t>YT coverage率</t>
+          <t>YT充足率</t>
         </is>
       </c>
       <c r="L1" t="inlineStr" s="1">
@@ -293,7 +293,7 @@
       </c>
       <c r="N1" t="inlineStr" s="1">
         <is>
-          <t>brand-only除外メモ</t>
+          <t>ブランド行除外メモ</t>
         </is>
       </c>
       <c r="O1" t="inlineStr" s="1">
@@ -360,7 +360,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -370,12 +370,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>model_id=NULL の brand-only 2件は denominator 外</t>
+          <t>model_id=NULL のブランド行2件は denominator 外</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>GTは一部0値あり。coverage gateは通過済み</t>
+          <t>GTは一部0値あり。充足ゲートは通過済み</t>
         </is>
       </c>
     </row>
@@ -402,27 +402,27 @@
       </c>
       <c r="C1" t="inlineStr" s="1">
         <is>
-          <t>kind</t>
+          <t>種別</t>
         </is>
       </c>
       <c r="D1" t="inlineStr" s="1">
         <is>
-          <t>candidate status</t>
+          <t>候補状態</t>
         </is>
       </c>
       <c r="E1" t="inlineStr" s="1">
         <is>
-          <t>promotable</t>
+          <t>公開可能</t>
         </is>
       </c>
       <c r="F1" t="inlineStr" s="1">
         <is>
-          <t>promotion実施</t>
+          <t>公開反映</t>
         </is>
       </c>
       <c r="G1" t="inlineStr" s="1">
         <is>
-          <t>release week</t>
+          <t>公開週</t>
         </is>
       </c>
       <c r="H1" t="inlineStr" s="1">
@@ -437,17 +437,17 @@
       </c>
       <c r="J1" t="inlineStr" s="1">
         <is>
-          <t>status確認</t>
+          <t>状態確認</t>
         </is>
       </c>
       <c r="K1" t="inlineStr" s="1">
         <is>
-          <t>stable markdown updated</t>
+          <t>安定版本文更新</t>
         </is>
       </c>
       <c r="L1" t="inlineStr" s="1">
         <is>
-          <t>issues</t>
+          <t>問題</t>
         </is>
       </c>
       <c r="M1" t="inlineStr" s="1">
@@ -469,22 +469,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ranking</t>
+          <t>ランキング</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>no_release</t>
+          <t>未公開</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>はい</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>はい</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -499,27 +499,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>確認済み</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>はい</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>なし</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>ranking release completed</t>
+          <t>ランキング release 完了</t>
         </is>
       </c>
     </row>
@@ -536,22 +536,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>compare</t>
+          <t>比較</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>no_release</t>
+          <t>未公開</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>はい</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>はい</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -566,27 +566,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>確認済み</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>はい</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>なし</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>compare release completed</t>
+          <t>比較 release 完了</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(training-trend-analyzer): add ranking dashboard view
</commit_message>
<xml_diff>
--- a/training-trend-analyzer/ops/publication_dashboard/publication_weekly_view.xlsx
+++ b/training-trend-analyzer/ops/publication_dashboard/publication_weekly_view.xlsx
@@ -5,6 +5,9 @@
     <sheet name="週次概要" sheetId="1" r:id="rId1"/>
     <sheet name="充足確認" sheetId="2" r:id="rId2"/>
     <sheet name="公開履歴" sheetId="3" r:id="rId3"/>
+    <sheet name="ランキング結果" sheetId="4" r:id="rId4"/>
+    <sheet name="ランキングの見方" sheetId="5" r:id="rId5"/>
+    <sheet name="ソース一覧" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -593,4 +596,1400 @@
   </sheetData>
   <autoFilter ref="A1:M3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:K12"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t>対象週</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t>順位</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t>機種名</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t>カテゴリ</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t>総合スコア</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
+          <t>GT値</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
+          <t>GS値</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr" s="1">
+        <is>
+          <t>YT値</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr" s="1">
+        <is>
+          <t>傾向コメント</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr" s="1">
+        <is>
+          <t>公開向けひとこと</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr" s="1">
+        <is>
+          <t>注意メモ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Concept2 SkiErg</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ski_erg</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>54.59</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>44.0</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>3.333</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>GTと補助ソースが揃い、今週の参考指標では最上位。</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Concept2 SkiErgは今週の検索系シグナルで上位候補です。</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>販売実績順位ではない。変化率は前週サポート条件によりN/A。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>TECHNOGYM Run</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>treadmill</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>54.25</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>58.0</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>GT値は高いが、総合スコアでは僅差で2位。</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>TECHNOGYM Runはトレッドミル領域で強い候補です。</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>1位との差は小さいため断定表現を避ける。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Life Fitness T5</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>treadmill</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>47.13</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>35.0</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>GT / GS / YT が揃い、上位候補として安定している。</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Life Fitness T5は今週の上位トレッドミル候補です。</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>変化率は前週サポート条件によりN/A。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Precor TRM 445</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>treadmill</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>39.37</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>26.0</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>GTとYTはあるが、GSはスコア計算上の最小値条件で除外。</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Precor TRM 445は参考候補として確認対象です。</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>GS値が低く、スコア上は一部除外扱い。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CYBEX 770T</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>treadmill</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>15.28</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>GSはあるがGT値が低く、信号の強さは慎重に見る。</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>CYBEX 770Tは補助ソース上の反応を確認する候補です。</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>GT値が低い。公開時は強い表現を避ける。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Life Fitness IC7</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>spin_bike</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>13.45</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>7.0</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>5.5</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>GS / YT はあるがGTは0値。</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Life Fitness IC7は補助ソース上で確認できる候補です。</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>GTが0値。検索トレンドとしては慎重に扱う。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Concept2 Model D</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>rowing</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>13.45</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>5.5</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>GS / YT はあるがGTは0値。</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Concept2 Model Dは補助ソース上で確認できる候補です。</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>GTが0値。検索トレンドとしては慎重に扱う。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Life Fitness 95T</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>treadmill</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>13.45</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>7.0</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>GS / YT はあるがGTは0値。</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Life Fitness 95Tは補助ソース上で確認できる候補です。</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>GTが0値。検索トレンドとしては慎重に扱う。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Life Fitness IC5</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>spin_bike</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>12.85</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>5.5</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>GS / YT はあるがGTは0値。</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Life Fitness IC5は補助ソース上で確認できる候補です。</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>GTが0値。検索トレンドとしては慎重に扱う。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Matrix A50</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>elliptical</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>12.03</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>GS / YT はあるがGTは0値。</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Matrix A50は補助ソース上で確認できる候補です。</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>GTが0値。検索トレンドとしては慎重に扱う。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>TECHNOGYM Run Now</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>treadmill</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>12.03</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>7.0</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>GS / YT はあるがGTは0値。</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>TECHNOGYM Run Nowは補助ソース上で確認できる候補です。</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>GTが0値。検索トレンドとしては慎重に扱う。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:K12"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t>区分</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t>項目</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t>説明</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>このランキングは何か</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>位置づけ</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>複数の検索系シグナルをもとに週次で整理した参考指標です。販売実績順位ではなく、公開判断を補助する運用ビューです。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>何をもとにしているか</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>使用ソース</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GT = Google Trends、GS = Google Suggest、YT = YouTube Suggest を使います。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>順位の考え方</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>複数ソースの総合</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>GT / GS / YT をまとめて見た総合スコアで並べます。単一ソースだけの人気順位ではありません。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>向いている見方</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>週次比較</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>同じルールで毎週見れば、上位候補や信号の変化を追いやすくなります。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>注意点</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>販売確定ではない</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>上位にあることは販売実績や導入実績の確定を意味しません。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>注意点</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>coverage gate の限界</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>coverage gate 通過は必要なソースが揃ったという意味であり、そのまま品質保証ではありません。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>注意点</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>低値 / 0値</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>GTの低値や0値は signal quality に注意し、公開文では断定しすぎないようにします。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>注意点</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>一時的な影響</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>一時的な話題性、検索語の揺れ、サジェストの特性によって順位や値が動くことがあります。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>信頼性の見せ方</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>根拠表示</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>使用ソース、対象週、正本の所在を明示します。正本は repo / Markdown / data/output / PROJECT_STATUS.md です。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Web公開時の注記</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>参考指標</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>本ランキングは、複数の検索系シグナルをもとに週次で整理した参考指標です。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Web公開時の注記</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>販売実績ではない</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>販売実績順位ではありません。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Web公開時の注記</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>変動可能性</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>公開時点のデータに基づくため、今後変動する可能性があります。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>再開時に見る場所</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>確認順</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>まず `ランキング結果` で今週の上位を見て、`ソース一覧` と `ランキングの見方` で根拠と注意点を確認します。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C14"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t>対象週</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t>機種名</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t>GT元データ有無</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t>GS元データ有無</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t>YT元データ有無</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
+          <t>データメモ</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
+          <t>解釈注意</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Concept2 SkiErg</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>GT=44.0 / GS=3.333 / YT=3.0</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>変化率は前週サポート条件によりN/A。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TECHNOGYM Run</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>GT=58.0 / GS=3.5 / YT=2.5</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>1位との差が小さいため断定しすぎない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Life Fitness T5</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>GT=35.0 / GS=4.0 / YT=3.0</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>変化率は前週サポート条件によりN/A。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Precor TRM 445</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>GT=26.0 / GS=1.5 / YT=2.0</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>GSは取得済みだがスコア計算上は value&lt;2 で除外。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CYBEX 770T</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>GT=4.0 / GS=9.0 / YT=3.0</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>GT値が低い。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Life Fitness IC7</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>GT=0.0 / GS=7.0 / YT=5.5</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>GTが0値。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Concept2 Model D</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>GT=0.0 / GS=9.0 / YT=5.5</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>GTが0値。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Life Fitness 95T</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>GT=0.0 / GS=9.0 / YT=7.0</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>GTが0値。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Life Fitness IC5</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>GT=0.0 / GS=6.0 / YT=5.5</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>GTが0値。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Matrix A50</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>GT=0.0 / GS=9.0 / YT=3.0</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>GTが0値。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>TECHNOGYM Run Now</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>GT=0.0 / GS=7.0 / YT=3.0</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>GTが0値。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G12"/>
+</worksheet>
 </file>
</xml_diff>